<commit_message>
docs: keep only single branch P-Block-Negative-Cases in platform matrix
</commit_message>
<xml_diff>
--- a/Platform_Stack_Matrix.xlsx
+++ b/Platform_Stack_Matrix.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -512,55 +512,28 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="42" customHeight="1">
+    <row r="2" ht="45" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>CE-CS-001</t>
+          <t>P-Block-Negative-Cases</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>C# / .NET 8.0 (LTS)</t>
+          <t>C# / .NET 9.0 &amp; JavaScript (ReactJS)</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>dotnet + NuGet</t>
+          <t>dotnet + NuGet &amp; Vite (esbuild) + npm</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Monolith</t>
+          <t>MVC (Model-View-Controller)</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>C# ASP.NET Core gRPC Server &amp; Client + Mongo + Angular single solution. Monolithic .NET 8 solution with unified project references.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="42" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>P-Block-Negative-Cases</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>C# / .NET 9.0 &amp; JavaScript (ReactJS)</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>dotnet + NuGet &amp; Vite (esbuild) + npm</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>MVC (Model-View-Controller)</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>C# ASP.NET Core Web API + SQL Server (EF Core) + ReactJS single solution. 9-Box talent matrix evaluation platform with negative and boundary test case validations.</t>
         </is>

</xml_diff>